<commit_message>
Update evaluation results using macro average in scores
</commit_message>
<xml_diff>
--- a/results/evaluation/evaluation_models.xlsx
+++ b/results/evaluation/evaluation_models.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nikos/UniPi/theses/langchain-encryption-feature/results/evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07AE7ABA-4D70-B34D-B1C0-DD35CBA8A8B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686F8A63-F411-6D46-802C-7896363FAB33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="mistral_plain" sheetId="1" r:id="rId1"/>

</xml_diff>